<commit_message>
Add More Info link and Team Members section to event drawer
- Extract URL from Headline column HTML and show as 'More Info ↗' after description
- Parse Team Members (Role: Name; format) into formatted section with underlined roles
- Add Research Team section label; space between role groups

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/timeline-data/IIF-Timeline-Data-Multi-Project.xlsx
+++ b/data/timeline-data/IIF-Timeline-Data-Multi-Project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasonlocal/Documents/Coding-Experiments/Timeline/Timeline-JEL/data/timeline-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5372885C-6DBE-6C45-B426-5632BDC2A502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4951DB76-D674-8A49-83B4-12AE32575A80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5580" yWindow="2300" windowWidth="29320" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6393,9 +6393,6 @@
     <t>2013</t>
   </si>
   <si>
-    <t>&lt;a href="http://skins.abtec.org/skins4.0/"&gt;Skins 4.0&lt;/a&gt;</t>
-  </si>
-  <si>
     <t>Skins 4.0</t>
   </si>
   <si>
@@ -6767,6 +6764,9 @@
   </si>
   <si>
     <t>The 4th installment of our intensive videogame workshops, this time for 3 weeks. Held at Concordia University with Indigenous youth, middles, and elders from Kahnawake.</t>
+  </si>
+  <si>
+    <t>&lt;a href="https://skins.abtec.org/skins4.0/"&gt;Skins 4.0&lt;/a&gt;</t>
   </si>
 </sst>
 </file>
@@ -8288,7 +8288,7 @@
         <v>20</v>
       </c>
       <c r="V1" s="5" t="s">
-        <v>2128</v>
+        <v>2127</v>
       </c>
       <c r="W1" s="5" t="s">
         <v>21</v>
@@ -34525,22 +34525,22 @@
       </c>
       <c r="H526" s="9"/>
       <c r="I526" s="9"/>
-      <c r="J526" s="101" t="s">
+      <c r="J526" s="19" t="s">
+        <v>2130</v>
+      </c>
+      <c r="K526" s="61" t="s">
         <v>2007</v>
       </c>
-      <c r="K526" s="61" t="s">
-        <v>2008</v>
-      </c>
       <c r="L526" s="7" t="s">
-        <v>2130</v>
+        <v>2129</v>
       </c>
       <c r="M526" s="114" t="s">
-        <v>2127</v>
+        <v>2126</v>
       </c>
       <c r="N526" s="7"/>
       <c r="O526" s="7"/>
       <c r="P526" s="7" t="s">
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="Q526" s="7"/>
       <c r="R526" s="7" t="s">
@@ -34556,7 +34556,7 @@
         <v>68</v>
       </c>
       <c r="V526" s="15" t="s">
-        <v>2129</v>
+        <v>2128</v>
       </c>
       <c r="W526" s="16" t="s">
         <v>30</v>
@@ -34580,18 +34580,18 @@
       <c r="H527" s="9"/>
       <c r="I527" s="9"/>
       <c r="J527" s="7" t="s">
+        <v>2009</v>
+      </c>
+      <c r="K527" s="61" t="s">
         <v>2010</v>
       </c>
-      <c r="K527" s="61" t="s">
+      <c r="L527" s="7" t="s">
         <v>2011</v>
-      </c>
-      <c r="L527" s="7" t="s">
-        <v>2012</v>
       </c>
       <c r="N527" s="7"/>
       <c r="O527" s="7"/>
       <c r="P527" s="7" t="s">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="Q527" s="7"/>
       <c r="R527" s="7" t="s">
@@ -34627,19 +34627,19 @@
       <c r="H528" s="9"/>
       <c r="I528" s="9"/>
       <c r="J528" s="7" t="s">
+        <v>2013</v>
+      </c>
+      <c r="K528" s="61" t="s">
         <v>2014</v>
       </c>
-      <c r="K528" s="61" t="s">
+      <c r="L528" s="7" t="s">
         <v>2015</v>
-      </c>
-      <c r="L528" s="7" t="s">
-        <v>2016</v>
       </c>
       <c r="M528" s="14"/>
       <c r="N528" s="7"/>
       <c r="O528" s="7"/>
       <c r="P528" s="7" t="s">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="Q528" s="7"/>
       <c r="R528" s="7" t="s">
@@ -34675,19 +34675,19 @@
       <c r="H529" s="9"/>
       <c r="I529" s="9"/>
       <c r="J529" s="7" t="s">
+        <v>2017</v>
+      </c>
+      <c r="K529" s="61" t="s">
         <v>2018</v>
       </c>
-      <c r="K529" s="61" t="s">
+      <c r="L529" s="7" t="s">
         <v>2019</v>
-      </c>
-      <c r="L529" s="7" t="s">
-        <v>2020</v>
       </c>
       <c r="M529" s="19"/>
       <c r="N529" s="7"/>
       <c r="O529" s="7"/>
       <c r="P529" s="7" t="s">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="Q529" s="7"/>
       <c r="R529" s="7" t="s">
@@ -34723,19 +34723,19 @@
       <c r="H530" s="9"/>
       <c r="I530" s="9"/>
       <c r="J530" s="101" t="s">
+        <v>2021</v>
+      </c>
+      <c r="K530" s="61" t="s">
         <v>2022</v>
       </c>
-      <c r="K530" s="61" t="s">
+      <c r="L530" s="7" t="s">
         <v>2023</v>
-      </c>
-      <c r="L530" s="7" t="s">
-        <v>2024</v>
       </c>
       <c r="M530" s="14"/>
       <c r="N530" s="7"/>
       <c r="O530" s="7"/>
       <c r="P530" s="7" t="s">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="Q530" s="7"/>
       <c r="R530" s="7" t="s">
@@ -34771,19 +34771,19 @@
       <c r="H531" s="9"/>
       <c r="I531" s="9"/>
       <c r="J531" s="7" t="s">
+        <v>2025</v>
+      </c>
+      <c r="K531" s="61" t="s">
         <v>2026</v>
       </c>
-      <c r="K531" s="61" t="s">
+      <c r="L531" s="7" t="s">
         <v>2027</v>
-      </c>
-      <c r="L531" s="7" t="s">
-        <v>2028</v>
       </c>
       <c r="M531" s="19"/>
       <c r="N531" s="7"/>
       <c r="O531" s="7"/>
       <c r="P531" s="7" t="s">
-        <v>2029</v>
+        <v>2028</v>
       </c>
       <c r="Q531" s="7"/>
       <c r="R531" s="7" t="s">
@@ -34819,19 +34819,19 @@
       <c r="H532" s="9"/>
       <c r="I532" s="9"/>
       <c r="J532" s="7" t="s">
+        <v>2029</v>
+      </c>
+      <c r="K532" s="61" t="s">
         <v>2030</v>
       </c>
-      <c r="K532" s="61" t="s">
+      <c r="L532" s="7" t="s">
         <v>2031</v>
-      </c>
-      <c r="L532" s="7" t="s">
-        <v>2032</v>
       </c>
       <c r="M532" s="19"/>
       <c r="N532" s="7"/>
       <c r="O532" s="7"/>
       <c r="P532" s="7" t="s">
-        <v>2033</v>
+        <v>2032</v>
       </c>
       <c r="Q532" s="7"/>
       <c r="R532" s="7" t="s">
@@ -34867,19 +34867,19 @@
       <c r="H533" s="9"/>
       <c r="I533" s="9"/>
       <c r="J533" s="7" t="s">
+        <v>2033</v>
+      </c>
+      <c r="K533" s="61" t="s">
         <v>2034</v>
       </c>
-      <c r="K533" s="61" t="s">
+      <c r="L533" s="7" t="s">
         <v>2035</v>
-      </c>
-      <c r="L533" s="7" t="s">
-        <v>2036</v>
       </c>
       <c r="M533" s="19"/>
       <c r="N533" s="7"/>
       <c r="O533" s="7"/>
       <c r="P533" s="7" t="s">
-        <v>2037</v>
+        <v>2036</v>
       </c>
       <c r="Q533" s="7"/>
       <c r="R533" s="7" t="s">
@@ -34921,13 +34921,13 @@
       <c r="H534" s="9"/>
       <c r="I534" s="9"/>
       <c r="J534" s="7" t="s">
+        <v>2037</v>
+      </c>
+      <c r="K534" s="61" t="s">
         <v>2038</v>
       </c>
-      <c r="K534" s="61" t="s">
+      <c r="L534" s="7" t="s">
         <v>2039</v>
-      </c>
-      <c r="L534" s="7" t="s">
-        <v>2040</v>
       </c>
       <c r="M534" s="7"/>
       <c r="N534" s="7"/>
@@ -34973,13 +34973,13 @@
       <c r="H535" s="9"/>
       <c r="I535" s="9"/>
       <c r="J535" s="7" t="s">
+        <v>2040</v>
+      </c>
+      <c r="K535" s="61" t="s">
         <v>2041</v>
       </c>
-      <c r="K535" s="61" t="s">
+      <c r="L535" s="7" t="s">
         <v>2042</v>
-      </c>
-      <c r="L535" s="7" t="s">
-        <v>2043</v>
       </c>
       <c r="M535" s="7"/>
       <c r="N535" s="7"/>
@@ -35019,13 +35019,13 @@
       <c r="H536" s="9"/>
       <c r="I536" s="9"/>
       <c r="J536" s="7" t="s">
-        <v>2044</v>
+        <v>2043</v>
       </c>
       <c r="K536" s="61" t="s">
         <v>1818</v>
       </c>
       <c r="L536" s="7" t="s">
-        <v>2045</v>
+        <v>2044</v>
       </c>
       <c r="M536" s="7"/>
       <c r="N536" s="7"/>
@@ -35071,13 +35071,13 @@
       <c r="H537" s="9"/>
       <c r="I537" s="9"/>
       <c r="J537" s="7" t="s">
+        <v>2045</v>
+      </c>
+      <c r="K537" s="61" t="s">
         <v>2046</v>
       </c>
-      <c r="K537" s="61" t="s">
-        <v>2047</v>
-      </c>
       <c r="L537" s="7" t="s">
-        <v>2043</v>
+        <v>2042</v>
       </c>
       <c r="M537" s="7"/>
       <c r="N537" s="7"/>
@@ -35117,21 +35117,21 @@
       <c r="H538" s="9"/>
       <c r="I538" s="9"/>
       <c r="J538" s="7" t="s">
+        <v>2047</v>
+      </c>
+      <c r="K538" s="61" t="s">
         <v>2048</v>
       </c>
-      <c r="K538" s="61" t="s">
+      <c r="L538" s="7" t="s">
         <v>2049</v>
-      </c>
-      <c r="L538" s="7" t="s">
-        <v>2050</v>
       </c>
       <c r="M538" s="14"/>
       <c r="N538" s="7" t="s">
-        <v>2052</v>
+        <v>2051</v>
       </c>
       <c r="O538" s="7"/>
       <c r="P538" s="7" t="s">
-        <v>2051</v>
+        <v>2050</v>
       </c>
       <c r="Q538" s="7"/>
       <c r="R538" s="7" t="s">
@@ -35173,19 +35173,19 @@
       <c r="H539" s="9"/>
       <c r="I539" s="9"/>
       <c r="J539" s="101" t="s">
+        <v>2052</v>
+      </c>
+      <c r="K539" s="61" t="s">
         <v>2053</v>
       </c>
-      <c r="K539" s="61" t="s">
+      <c r="L539" s="7" t="s">
         <v>2054</v>
-      </c>
-      <c r="L539" s="7" t="s">
-        <v>2055</v>
       </c>
       <c r="M539" s="14"/>
       <c r="N539" s="7"/>
       <c r="O539" s="7"/>
       <c r="P539" s="7" t="s">
-        <v>2056</v>
+        <v>2055</v>
       </c>
       <c r="Q539" s="7"/>
       <c r="R539" s="7" t="s">
@@ -35227,19 +35227,19 @@
       <c r="H540" s="9"/>
       <c r="I540" s="9"/>
       <c r="J540" s="101" t="s">
+        <v>2056</v>
+      </c>
+      <c r="K540" s="61" t="s">
         <v>2057</v>
       </c>
-      <c r="K540" s="61" t="s">
+      <c r="L540" s="7" t="s">
         <v>2058</v>
-      </c>
-      <c r="L540" s="7" t="s">
-        <v>2059</v>
       </c>
       <c r="M540" s="19"/>
       <c r="N540" s="7"/>
       <c r="O540" s="7"/>
       <c r="P540" s="7" t="s">
-        <v>2060</v>
+        <v>2059</v>
       </c>
       <c r="Q540" s="18"/>
       <c r="R540" s="7" t="s">
@@ -35281,13 +35281,13 @@
       <c r="H541" s="9"/>
       <c r="I541" s="9"/>
       <c r="J541" s="101" t="s">
+        <v>2060</v>
+      </c>
+      <c r="K541" s="61" t="s">
         <v>2061</v>
       </c>
-      <c r="K541" s="61" t="s">
-        <v>2062</v>
-      </c>
       <c r="L541" s="7" t="s">
-        <v>2059</v>
+        <v>2058</v>
       </c>
       <c r="M541" s="7"/>
       <c r="N541" s="7"/>
@@ -35327,13 +35327,13 @@
       <c r="H542" s="9"/>
       <c r="I542" s="9"/>
       <c r="J542" s="101" t="s">
+        <v>2062</v>
+      </c>
+      <c r="K542" s="61" t="s">
         <v>2063</v>
       </c>
-      <c r="K542" s="61" t="s">
+      <c r="L542" s="7" t="s">
         <v>2064</v>
-      </c>
-      <c r="L542" s="7" t="s">
-        <v>2065</v>
       </c>
       <c r="M542" s="7"/>
       <c r="N542" s="7"/>
@@ -35373,13 +35373,13 @@
       <c r="H543" s="9"/>
       <c r="I543" s="9"/>
       <c r="J543" s="101" t="s">
+        <v>2065</v>
+      </c>
+      <c r="K543" s="61" t="s">
         <v>2066</v>
       </c>
-      <c r="K543" s="61" t="s">
+      <c r="L543" s="7" t="s">
         <v>2067</v>
-      </c>
-      <c r="L543" s="7" t="s">
-        <v>2068</v>
       </c>
       <c r="M543" s="7"/>
       <c r="N543" s="7"/>
@@ -35419,13 +35419,13 @@
       <c r="H544" s="9"/>
       <c r="I544" s="9"/>
       <c r="J544" s="101" t="s">
+        <v>2068</v>
+      </c>
+      <c r="K544" s="61" t="s">
         <v>2069</v>
       </c>
-      <c r="K544" s="61" t="s">
+      <c r="L544" s="7" t="s">
         <v>2070</v>
-      </c>
-      <c r="L544" s="7" t="s">
-        <v>2071</v>
       </c>
       <c r="M544" s="7"/>
       <c r="N544" s="7"/>
@@ -35471,19 +35471,19 @@
       <c r="H545" s="9"/>
       <c r="I545" s="9"/>
       <c r="J545" s="101" t="s">
+        <v>2071</v>
+      </c>
+      <c r="K545" s="61" t="s">
         <v>2072</v>
       </c>
-      <c r="K545" s="61" t="s">
+      <c r="L545" s="7" t="s">
         <v>2073</v>
-      </c>
-      <c r="L545" s="7" t="s">
-        <v>2074</v>
       </c>
       <c r="M545" s="19"/>
       <c r="N545" s="7"/>
       <c r="O545" s="7"/>
       <c r="P545" s="107" t="s">
-        <v>2075</v>
+        <v>2074</v>
       </c>
       <c r="Q545" s="7"/>
       <c r="R545" s="7" t="s">
@@ -35525,19 +35525,19 @@
       <c r="H546" s="9"/>
       <c r="I546" s="9"/>
       <c r="J546" s="101" t="s">
+        <v>2075</v>
+      </c>
+      <c r="K546" s="61" t="s">
         <v>2076</v>
       </c>
-      <c r="K546" s="61" t="s">
+      <c r="L546" s="7" t="s">
         <v>2077</v>
-      </c>
-      <c r="L546" s="7" t="s">
-        <v>2078</v>
       </c>
       <c r="M546" s="19"/>
       <c r="N546" s="7"/>
       <c r="O546" s="7"/>
       <c r="P546" s="7" t="s">
-        <v>2079</v>
+        <v>2078</v>
       </c>
       <c r="Q546" s="7"/>
       <c r="R546" s="7" t="s">
@@ -35573,19 +35573,19 @@
       <c r="H547" s="9"/>
       <c r="I547" s="9"/>
       <c r="J547" s="101" t="s">
+        <v>2079</v>
+      </c>
+      <c r="K547" s="61" t="s">
         <v>2080</v>
       </c>
-      <c r="K547" s="61" t="s">
+      <c r="L547" s="7" t="s">
         <v>2081</v>
-      </c>
-      <c r="L547" s="7" t="s">
-        <v>2082</v>
       </c>
       <c r="M547" s="14"/>
       <c r="N547" s="7"/>
       <c r="O547" s="7"/>
       <c r="P547" s="7" t="s">
-        <v>2083</v>
+        <v>2082</v>
       </c>
       <c r="Q547" s="7"/>
       <c r="R547" s="7" t="s">
@@ -35627,19 +35627,19 @@
       <c r="H548" s="9"/>
       <c r="I548" s="9"/>
       <c r="J548" s="101" t="s">
+        <v>2083</v>
+      </c>
+      <c r="K548" s="61" t="s">
         <v>2084</v>
       </c>
-      <c r="K548" s="61" t="s">
+      <c r="L548" s="7" t="s">
         <v>2085</v>
-      </c>
-      <c r="L548" s="7" t="s">
-        <v>2086</v>
       </c>
       <c r="M548" s="19"/>
       <c r="N548" s="7"/>
       <c r="O548" s="7"/>
       <c r="P548" s="7" t="s">
-        <v>2087</v>
+        <v>2086</v>
       </c>
       <c r="Q548" s="7"/>
       <c r="R548" s="7" t="s">
@@ -35675,19 +35675,19 @@
       <c r="H549" s="9"/>
       <c r="I549" s="9"/>
       <c r="J549" s="101" t="s">
+        <v>2087</v>
+      </c>
+      <c r="K549" s="61" t="s">
         <v>2088</v>
       </c>
-      <c r="K549" s="61" t="s">
+      <c r="L549" s="7" t="s">
         <v>2089</v>
-      </c>
-      <c r="L549" s="7" t="s">
-        <v>2090</v>
       </c>
       <c r="M549" s="14"/>
       <c r="N549" s="7"/>
       <c r="O549" s="7"/>
       <c r="P549" s="7" t="s">
-        <v>2091</v>
+        <v>2090</v>
       </c>
       <c r="Q549" s="7"/>
       <c r="R549" s="7" t="s">
@@ -35718,7 +35718,7 @@
       </c>
       <c r="D550" s="9"/>
       <c r="E550" s="9" t="s">
-        <v>2092</v>
+        <v>2091</v>
       </c>
       <c r="F550" s="9" t="s">
         <v>145</v>
@@ -35729,13 +35729,13 @@
       <c r="H550" s="9"/>
       <c r="I550" s="9"/>
       <c r="J550" s="7" t="s">
+        <v>2092</v>
+      </c>
+      <c r="K550" s="61" t="s">
         <v>2093</v>
       </c>
-      <c r="K550" s="61" t="s">
+      <c r="L550" s="7" t="s">
         <v>2094</v>
-      </c>
-      <c r="L550" s="7" t="s">
-        <v>2095</v>
       </c>
       <c r="M550" s="7"/>
       <c r="N550" s="7"/>
@@ -35781,13 +35781,13 @@
       <c r="H551" s="9"/>
       <c r="I551" s="9"/>
       <c r="J551" s="101" t="s">
+        <v>2095</v>
+      </c>
+      <c r="K551" s="61" t="s">
         <v>2096</v>
       </c>
-      <c r="K551" s="61" t="s">
+      <c r="L551" s="7" t="s">
         <v>2097</v>
-      </c>
-      <c r="L551" s="7" t="s">
-        <v>2098</v>
       </c>
       <c r="M551" s="7"/>
       <c r="N551" s="7"/>
@@ -35827,19 +35827,19 @@
       <c r="H552" s="9"/>
       <c r="I552" s="9"/>
       <c r="J552" s="101" t="s">
+        <v>2098</v>
+      </c>
+      <c r="K552" s="61" t="s">
         <v>2099</v>
       </c>
-      <c r="K552" s="61" t="s">
+      <c r="L552" s="7" t="s">
         <v>2100</v>
-      </c>
-      <c r="L552" s="7" t="s">
-        <v>2101</v>
       </c>
       <c r="M552" s="14"/>
       <c r="N552" s="7"/>
       <c r="O552" s="7"/>
       <c r="P552" s="7" t="s">
-        <v>2102</v>
+        <v>2101</v>
       </c>
       <c r="Q552" s="7"/>
       <c r="R552" s="7" t="s">
@@ -35875,13 +35875,13 @@
       <c r="H553" s="9"/>
       <c r="I553" s="9"/>
       <c r="J553" s="7" t="s">
+        <v>2102</v>
+      </c>
+      <c r="K553" s="61" t="s">
         <v>2103</v>
       </c>
-      <c r="K553" s="61" t="s">
-        <v>2104</v>
-      </c>
       <c r="L553" s="7" t="s">
-        <v>2101</v>
+        <v>2100</v>
       </c>
       <c r="M553" s="7"/>
       <c r="N553" s="7"/>
@@ -52906,7 +52906,7 @@
     <hyperlink ref="J522" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000031020000}"/>
     <hyperlink ref="J523" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000033020000}"/>
     <hyperlink ref="J524" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000035020000}"/>
-    <hyperlink ref="J526" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000038020000}"/>
+    <hyperlink ref="J526" r:id="rId71" display="&lt;a href=&quot;http://skins.abtec.org/skins4.0/&quot;&gt;Skins 4.0&lt;/a&gt;" xr:uid="{00000000-0004-0000-0000-000038020000}"/>
     <hyperlink ref="J530" r:id="rId72" xr:uid="{00000000-0004-0000-0000-00003D020000}"/>
     <hyperlink ref="J539" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000043020000}"/>
     <hyperlink ref="J540" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000045020000}"/>
@@ -52951,13 +52951,13 @@
         <v>18</v>
       </c>
       <c r="E1" s="25" t="s">
+        <v>2104</v>
+      </c>
+      <c r="G1" s="25" t="s">
         <v>2105</v>
       </c>
-      <c r="G1" s="25" t="s">
+      <c r="I1" s="25" t="s">
         <v>2106</v>
-      </c>
-      <c r="I1" s="25" t="s">
-        <v>2107</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="14" customHeight="1">
@@ -52968,7 +52968,7 @@
         <v>26</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>2108</v>
+        <v>2107</v>
       </c>
       <c r="G2" s="25" t="s">
         <v>140</v>
@@ -52979,64 +52979,64 @@
     </row>
     <row r="3" spans="1:9" ht="14" customHeight="1">
       <c r="A3" s="25" t="s">
+        <v>2108</v>
+      </c>
+      <c r="C3" s="25" t="s">
         <v>2109</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="E3" s="25" t="s">
         <v>2110</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>2111</v>
       </c>
       <c r="G3" s="25" t="s">
         <v>38</v>
       </c>
       <c r="I3" s="25" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="14" customHeight="1">
       <c r="A4" s="25" t="s">
+        <v>2112</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="25" t="s">
         <v>2113</v>
       </c>
-      <c r="C4" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="25" t="s">
+      <c r="G4" s="25" t="s">
         <v>2114</v>
       </c>
-      <c r="G4" s="25" t="s">
+      <c r="I4" s="25" t="s">
         <v>2115</v>
-      </c>
-      <c r="I4" s="25" t="s">
-        <v>2116</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="14" customHeight="1">
       <c r="C5" s="25" t="s">
-        <v>2117</v>
+        <v>2116</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>2115</v>
+        <v>2114</v>
       </c>
       <c r="G5" s="25" t="s">
         <v>286</v>
       </c>
       <c r="I5" s="25" t="s">
-        <v>2118</v>
+        <v>2117</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="14" customHeight="1">
       <c r="C6" s="25" t="s">
+        <v>2118</v>
+      </c>
+      <c r="E6" s="25" t="s">
         <v>2119</v>
-      </c>
-      <c r="E6" s="25" t="s">
-        <v>2120</v>
       </c>
       <c r="G6" s="25" t="s">
         <v>276</v>
       </c>
       <c r="I6" s="25" t="s">
-        <v>2121</v>
+        <v>2120</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="14" customHeight="1">
@@ -53054,7 +53054,7 @@
     <row r="8" spans="1:9" ht="14" customHeight="1">
       <c r="C8" s="25"/>
       <c r="E8" s="25" t="s">
-        <v>2122</v>
+        <v>2121</v>
       </c>
       <c r="G8" s="25" t="s">
         <v>136</v>
@@ -53063,7 +53063,7 @@
     </row>
     <row r="9" spans="1:9" ht="14" customHeight="1">
       <c r="E9" s="25" t="s">
-        <v>2123</v>
+        <v>2122</v>
       </c>
       <c r="G9" s="25" t="s">
         <v>108</v>
@@ -53072,7 +53072,7 @@
     </row>
     <row r="10" spans="1:9" ht="14" customHeight="1">
       <c r="E10" s="25" t="s">
-        <v>2124</v>
+        <v>2123</v>
       </c>
       <c r="G10" s="25" t="s">
         <v>68</v>
@@ -53081,7 +53081,7 @@
     </row>
     <row r="11" spans="1:9" ht="14" customHeight="1">
       <c r="E11" s="25" t="s">
-        <v>2125</v>
+        <v>2124</v>
       </c>
       <c r="G11" s="25"/>
       <c r="I11" s="25"/>
@@ -53093,7 +53093,7 @@
     </row>
     <row r="13" spans="1:9" ht="14" customHeight="1">
       <c r="E13" s="25" t="s">
-        <v>2126</v>
+        <v>2125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>